<commit_message>
update the headcount estimator
</commit_message>
<xml_diff>
--- a/data/ROSA/HEADCOUNT_TEMPLATE_ROSA.xlsx
+++ b/data/ROSA/HEADCOUNT_TEMPLATE_ROSA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10909"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WTK_TestPlaner\data\ROSA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/victor/Desktop/TestPlaner/WTK_TestPlaner/data/ROSA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{736E74E7-AF9B-43CC-8C7A-4C38DAA29BA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72C109DF-5655-CD40-ADF4-796845E144F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,15 +29,37 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="8">
+  <si>
+    <t xml:space="preserve">Phase </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month </t>
+  </si>
+  <si>
+    <t>Concept</t>
+  </si>
+  <si>
+    <t>BU</t>
+  </si>
+  <si>
+    <t>NOT</t>
+  </si>
+  <si>
+    <t>Structure Engineer</t>
+  </si>
+  <si>
+    <t>CAE Engineer</t>
+  </si>
+  <si>
+    <t>S&amp;V Engineer</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -46,13 +68,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="新細明體"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
@@ -82,7 +104,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -360,9 +382,110 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A1:M5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" t="s">
+        <v>4</v>
+      </c>
+      <c r="M1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <v>7</v>
+      </c>
+      <c r="I2">
+        <v>8</v>
+      </c>
+      <c r="J2">
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <v>10</v>
+      </c>
+      <c r="L2">
+        <v>11</v>
+      </c>
+      <c r="M2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>